<commit_message>
Harden demo controls workbook
</commit_message>
<xml_diff>
--- a/demo_evidence/controls.xlsx
+++ b/demo_evidence/controls.xlsx
@@ -427,7 +427,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="37" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -461,12 +461,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Quarterly user access reviews are performed and retained.</t>
+          <t>Quarterly user access reviews are performed and documented.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Access review evidence</t>
+          <t>Policy document, Access review export, Meeting notes</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -483,12 +483,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Terminated user access is removed within 24 hours.</t>
+          <t>Terminated users have access removed within 24 hours.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Termination ticket or access export</t>
+          <t>Policy document, Ticket dump, User access export</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -505,12 +505,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Privileged access is approved and limited to authorized administrators.</t>
+          <t>Privileged or administrator access is reviewed and approved.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Admin access approval</t>
+          <t>User access export, Access review export, Meeting notes</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -527,12 +527,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Password standards require complexity, rotation, and lockout controls.</t>
+          <t>Password policy requirements are formally documented.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Access policy</t>
+          <t>Policy document</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -549,12 +549,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Production changes are documented in approved change tickets.</t>
+          <t>Application or infrastructure changes are logged through tickets.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Change ticket</t>
+          <t>Ticket dump</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -571,12 +571,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Emergency changes receive retrospective review and approval.</t>
+          <t>Changes are reviewed and approved before implementation.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Emergency change review</t>
+          <t>Ticket dump, Meeting notes</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -593,12 +593,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Change testing evidence is retained before implementation.</t>
+          <t>Emergency changes are documented after implementation.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Testing evidence</t>
+          <t>Ticket dump, Meeting notes</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -615,12 +615,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Segregation of duties is maintained between request, approval, and deployment.</t>
+          <t>Change records include implementation status and description.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Change approval log</t>
+          <t>Ticket dump</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -637,12 +637,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sensitive data is encrypted at rest in approved storage locations.</t>
+          <t>Sensitive or personal data handling requirements are documented.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Encryption configuration</t>
+          <t>Policy document, Meeting notes</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -659,12 +659,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Backups are monitored and restoration tests are performed periodically.</t>
+          <t>Access to sensitive data is restricted by role or access level.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Backup and restore evidence</t>
+          <t>User access export, Policy document</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -681,12 +681,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Firewall rules are reviewed for unnecessary inbound access.</t>
+          <t>Security incidents are tracked and reviewed.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Firewall rules export</t>
+          <t>Ticket dump, Meeting notes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Security incidents are tracked, triaged, and closed with documented resolution.</t>
+          <t>Firewall or network protection evidence is maintained.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Incident ticket</t>
+          <t>Firewall rules screenshot</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">

</xml_diff>